<commit_message>
Publish accreditation explorer and updated AIQ bond guidance
</commit_message>
<xml_diff>
--- a/exports/state-bond-comparison.xlsx
+++ b/exports/state-bond-comparison.xlsx
@@ -8,19 +8,21 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read first" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State comparison" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Institution exceptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Written checks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="College confirmation tracker" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCC AIQ years" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State comparison" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Institution exceptions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Written checks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="College confirmation tracker" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read first'!$A$1:$B$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'State comparison'!$A$1:$O$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Institution exceptions'!$A$1:$C$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Written checks'!$A$1:$B$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sources'!$A$1:$L$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'College confirmation tracker'!$A$1:$R$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read first'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MCC AIQ years'!$A$1:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'State comparison'!$A$1:$T$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Institution exceptions'!$A$1:$C$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Written checks'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sources'!$A$1:$L$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'College confirmation tracker'!$A$1:$R$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -460,36 +462,36 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Your MCC AIQ route</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Do not assume Delhi is free of post-PG service bonds. MAMC circular dated 7 August 2025 expressly introduces one year / Rs20 lakh for PG entrants from 2025–26 onwards, AIQ and state quota. DU's 2026 Rs10 lakh surety is a separate course-exit bond. Other Delhi campuses need their own current authority/cohort check.</t>
+          <t>MCC allotment does not waive an applicable service bond. Read the AIQ-specific years and evidence column first. In Andhra Pradesh, the checked one-year undertaking explicitly names State/CQ seats, so an AIQ duration remains unconfirmed. Delhi has no single duration: MAMC is one year from 2025–26 onwards; other campuses require their own rule.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Limits</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>A mixed-date evidence comparison, not a fully verified 2026 national bond schedule or a legal enforceability opinion. Unresolved terms remain unknown, never zero. Sources checked 18 October 2026; apply subsequent amendments.</t>
+          <t>Do not assume Delhi is free of post-PG service bonds. MAMC circular dated 7 August 2025 expressly introduces one year / Rs20 lakh for PG entrants from 2025–26 onwards, AIQ and state quota. DU's 2026 Rs10 lakh surety is a separate course-exit bond. Other Delhi campuses need their own current authority/cohort check.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Definition</t>
+          <t>Limits</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Service bond: work owed after successful completion. The quoted amount is a default liability, not an annual fee or a charge automatically payable by every graduate.</t>
+          <t>A mixed-date evidence comparison, not a fully verified 2026 national bond schedule or a legal enforceability opinion. Unresolved terms remain unknown, never zero. Sources checked 18 October 2026; apply subsequent amendments.</t>
         </is>
       </c>
     </row>
@@ -501,7 +503,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Exit bond: liability for non-joining, resignation or discontinuation at specified stages. This is separate from compulsory service and counselling security-deposit forfeiture.</t>
+          <t>Service bond: work owed after successful completion. The quoted amount is a default liability, not an annual fee or a charge automatically payable by every graduate.</t>
         </is>
       </c>
     </row>
@@ -513,7 +515,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>A bank guarantee or surety secures an obligation. Do not add it again to the underlying bond amount. Do not automatically add service and exit penalties; their triggers and interaction need the executed contract.</t>
+          <t>Exit bond: liability for non-joining, resignation or discontinuation at specified stages. This is separate from compulsory service and counselling security-deposit forfeiture.</t>
         </is>
       </c>
     </row>
@@ -525,7 +527,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>AIQ/MCC admission does not itself exempt a candidate from the admitting institution's applicable state service bond. Central/INI, private/deemed, state government and DNB contracts must be checked separately.</t>
+          <t>A bank guarantee or surety secures an obligation. Do not add it again to the underlying bond amount. Do not automatically add service and exit penalties; their triggers and interaction need the executed contract.</t>
         </is>
       </c>
     </row>
@@ -537,7 +539,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>This comparison concerns ordinary non-in-service MD/MS entrants unless a row says otherwise. Diploma, DNB/DrNB, direct six-year courses, sponsored and in-service obligations are not interchangeable.</t>
+          <t>AIQ/MCC admission does not itself exempt a candidate from the admitting institution's applicable state service bond. Central/INI, private/deemed, state government and DNB contracts must be checked separately.</t>
         </is>
       </c>
     </row>
@@ -549,12 +551,24 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>This comparison concerns ordinary non-in-service MD/MS entrants unless a row says otherwise. Diploma, DNB/DrNB, direct six-year courses, sponsored and in-service obligations are not interchangeable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
           <t>An old form, missing upload or silent prospectus is not proof of no bond. A checked 2026 rule is an admission-cycle snapshot, not a guarantee of the rule when a future graduate finishes.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -565,7 +579,699 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>preference</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>service_years_label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>service_years_in_cited_evidence</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>evidence_status</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>applicability_and_limits</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>1 year · confirm cohort</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Plan for one year if required at Gandhi/Osmania. Their MCC service forms are older; 2026 CQ rules corroborate the duration but do not by themselves settle all AIQ campuses.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700481&amp;Type=BM
+https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700483&amp;Type=BM
+https://www.knruhs.telangana.gov.in/wp-content/uploads/notifications/20261014110317_KNRUHS-MEDICAL-PG-DEGREE-DIPLOMA-ADMISSIONS-UNDER-COMPETENT-AUTHORITY-QUOTA-FOR-THE-AY-2026-27-PROSPECTUS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>AIQ not established</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>State/CQ scope only</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>The one-year / Rs40 lakh Annexure A explicitly covers State/CQ seats. Obtain the government-college AIQ undertaking; do not infer either one year or zero for AIQ.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>https://drntr.uhsap.in/index/notification/20261014153141837.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2 years</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Explicit AIQ: 2026 prospectus</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Government medical colleges, non-service MD/MS, explicitly including 50% AIQ; two years within three years if services required.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>https://tnmedicalselection.net/news/08102026235127.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>3 years · current order needed</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Older AIQ form + 2026 secondary report</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Government-subsidised seats including AIQ. Reported March 2026 order credits an already completed statutory year, leaving two additional years; do not add these as four. Obtain the operative order.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>https://medicaldialogues.in/pdf_upload/kea-bond-255589.pdf
+https://medicaldialogues.in/news/health/doctors/rs-50-lakh-penalty-3-year-govt-service-karnataka-pg-medical-bond-policy-167423</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Kerala</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>1 year minimum</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Explicit AIQ: 2026 prospectus</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Government medical-college AIQ explicitly included in clause 11-1(b); continuous SR service for not less than one year. Conditional appointment/SS relief is separate.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://cee.kerala.gov.in/pgm2026/pdf/Prospectus.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Goa</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>1 year · older rule</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Goa Medical College 2020 PG amendment uploaded on MCC changes three years to one. Current continuation and original rule’s AIQ scope require the current college contract.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700479&amp;Type=BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Explicit AIQ: 2026 prospectus</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Government/municipal colleges; clause 20.4 expressly includes All India PG quota. Private unaided prohibition and AFMS obligations have separate scopes.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://statecetcell.s3.ap-south-1.amazonaws.com/2026/PGM/PGM-26_IB.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>1 year · confirm cohort</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>GMC Bhopal MCC form: ordinary entrant one-year rural service. Form cites amendments through September 2025; confirm current college/year and private scope.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700296&amp;Type=BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>MAMC: 1 year; others vary</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Explicit AIQ: MAMC 2025–26 onwards</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>MAMC circular expressly includes AIQ and state quota. No uniform Delhi duration: UCMS, LHMC, VMMC, ABVIMS/RML need their own applicable policy.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://medicaldialogues.in/pdf_upload/1326200011-297479.pdf
+https://storage.googleapis.com/dudocsfmsc/1791803818376-1791371447114-BOI_2026.pdf
+https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700122&amp;Type=BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Odisha</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2 years · confirm cohort</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>SCB government-college bond supplied on MCC specifies two years; AIQ not separately named and year blank. January 2026 placement guidance corroborates two years for a graduating cohort.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700336&amp;Type=BM
+https://dmetodisha.in/POST_PG_Static/DOWNLOADSPGM_22/GUIDELINES FOR POST PG BOND SR DOCTORS_02_01_2026.pdf
+https://dmetodisha.in/PGMCC_Static/DOWNLOADSPGM_22/Guidelines-for-admission-of-candidates-for-post-graduate-medical-courses-in-govt-and-private-medical-college-of-state-2026-27.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Puducherry</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Campus / route unresolved</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Current AIQ terms unresolved</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Separate a genuine state-government MD/MS AIQ seat from deemed paid seats and DNB. JIPMER MD/MS is an INI-CET route outside this MCC AIQ table. No current universal zero-year finding.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Jharkhand</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>3 years · older rule</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>RIMS Ranchi MCC-uploaded 2018 resolution. Confirm current RIMS/other state-college AIQ contract; this is not a rule for central AIIMS Deoghar.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700418&amp;Type=BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Rajasthan</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2 years · confirm cohort</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Dr SN Jodhpur non-service form explicitly names AIQ. The page with five years is in-service. Values differ by branch; other campus/current relief orders require checking.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700308&amp;Type=BM
+https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700327&amp;Type=BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2 years · older rule</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>State government/autonomous colleges under the KGMU form citing the 2018 order. Central BHU/AMU, AIIMS and private/DNB are separate; geography does not transfer this bond.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700366&amp;Type=BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Uttarakhand</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2 years · scheme dependent</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Conditional subsidised-fee scheme</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Older undertaking expressly includes Central quota but links service to opting for subsidised tuition. Mixed Doon/Haldwani documents do not establish a universal current two-year obligation or exemption for full-fee seats.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700386&amp;Type=BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>3 years · confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Three years corroborated by 2026 open/non-service bulletin and Burdwan MCC bond. Confirm college AIQ cohort; open means non-in-service, not only UR reservation.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://cdnbbsr.s3waas.gov.in/s3aae8d1e00b15a30e5901227e97ffbef7/uploads/2026/10/2026101495338605.pdf
+https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700388&amp;Type=BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Chhattisgarh</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2 years · 2025 form</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Pt JNM Raipur form expressly includes AIQ/state, cites November 2025 gazette and fills admission year 2025. Confirm current form; do not apply to AIIMS Raipur.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700316&amp;Type=BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Bihar</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>3 years · 2025 prospectus</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>State-government PG bonds in 2025 prospectus. Specified already-government-employed AIQ entrants have a 2019 exception; ordinary AIQ admission alone is not that exception.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>https://bceceboard.bihar.gov.in/pdf_Pros/PROS_PGMAC25.pdf</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G19"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -583,6 +1289,11 @@
     <col width="42" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
     <col width="42" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="18" max="18"/>
+    <col width="42" customWidth="1" min="19" max="19"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -603,60 +1314,85 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>aiq_service_label</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>aiq_service_years</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>aiq_review_status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>aiq_scope_note</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>aiq_source_ids</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>evidence_status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>admission_cycle</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>applicability</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>service_years</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>service_requirement</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>service_default_principal_inr</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>service_default_terms</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>course_exit_terms</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>exceptions_and_in_service</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>higher_studies</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>posting_and_release</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>source_ids</t>
         </is>
@@ -680,58 +1416,81 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>1 year · confirm cohort</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Plan for one year if required at Gandhi/Osmania. Their MCC service forms are older; 2026 CQ rules corroborate the duration but do not by themselves settle all AIQ campuses.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700481-BM; mcc-700483-BM; ts-cq2026</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>2026 prospectus</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>2026–27 competent-authority admissions</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>KNRUHS competent-authority PG entrants; non-in-service service clause. Obtain separate AIQ/management/deemed/central/DNB applicability.</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>2026–27 competent-authority rule plus Gandhi/Osmania government-college bonds uploaded to MCC. College forms support AIQ planning but their 2025–26 / 2023–24 dates need updating.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>One year in Telangana government institutions, if required by government.</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="N2" s="2" t="n">
         <v>2000000</v>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>MD/MS degree bond Rs20 lakh; diploma Rs10 lakh is a different qualification.</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Rs50 lakh plus stipend/salary refund for failure to complete training; after free-exit date, Rs50 lakh and three-year KNRUHS PG counselling debarment stated separately.</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>In-service candidates have separate government-employment rules; not the default applicant category.</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Not established from the checked material; obtain the current college/order clause.</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>ts-cq2026</t>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>Gandhi 2025–26 form: one year as SR if required, completed within 18 months. This is a completion window, not a verified automatic release if no appointment is offered.</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>ts-cq2026; mcc-700481-BM; mcc-700483-BM</t>
         </is>
       </c>
     </row>
@@ -753,56 +1512,77 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>AIQ not established</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>State/CQ scope only</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>The one-year / Rs40 lakh Annexure A explicitly covers State/CQ seats. Obtain the government-college AIQ undertaking; do not infer either one year or zero for AIQ.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>ap-cq2026</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>2026 prospectus</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>2026–27 competent-authority admissions</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Section 5 non-service PG entrants in checked CQ prospectus; confirm exact college/quota. SVIMS has its own appended terms.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>2026–27 Annexure A explicitly names State Quota / Competent Authority seats in government/private colleges. It is not a verified AIQ service undertaking. SVIMS has separate terms.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>One year of service, completed within 18 months after obtaining the PG degree.</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="N3" s="2" t="n">
         <v>4000000</v>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>Rs40 lakh if not joining/completing the required service, citing GO251 of 2 October 2022.</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>MQ prospectus states Rs3 lakh plus stipend refund and three-year debarment. CQ exit clause has a PG Dental wording carryover; obtain the correct MD/MS form.</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>In-service: ten years; Rs50 lakh plus pay/allowances and applicable interest. Do not apply this to ordinary entrants. MQ exit terms do not prove MQ post-PG service.</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>In-service: ten years; Rs50 lakh plus pay/allowances and applicable interest. Do not apply this to ordinary entrants. MQ exit terms do not prove MQ post-PG service. For this applicant’s MCC AIQ route, do not assign one year or Rs40 lakh from the State/CQ-only Annexure A. Neither a separate AIQ obligation nor an explicit AIQ exemption is established here.</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>In-service SS deferment is described; ordinary-entrant SS/fellowship deferral not established.</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>18 months is a service-completion window, not a verified automatic-release deadline if no posting is offered.</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>ap-cq2026; ap-mq2026</t>
         </is>
@@ -826,56 +1606,79 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>2 years</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Explicit AIQ: 2026 prospectus</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Government medical colleges, non-service MD/MS, explicitly including 50% AIQ; two years within three years if services required.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>tn-gq2026</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
           <t>2026 prospectus</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>2026–27</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Non-service candidates joining government medical colleges, explicitly including 50% AIQ.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="L4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Two years within three years after PG completion, if government requires services.</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="N4" s="2" t="n">
         <v>4000000</v>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>Degree Rs40 lakh or proportionate unserved liability, plus specified interest from demand. Diploma Rs20 lakh separately.</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>Discontinuation fee under clause 24(c) plus stipend received; timing and amount must be checked separately.</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>In-service candidates: service until superannuation; a separate five-year rule applies when less than five years remain. Private/deemed seats are not automatically covered by this government-college row.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>Paid on par with fresh Tamil Nadu Medical Service recruits. Check posting, three-year window and written discharge; no guaranteed permanent appointment.</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>tn-gq2026</t>
         </is>
@@ -899,56 +1702,79 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>3 years · current order needed</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Older AIQ form + 2026 secondary report</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Government-subsidised seats including AIQ. Reported March 2026 order credits an already completed statutory year, leaving two additional years; do not add these as four. Obtain the operative order.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>kar-kea-forms2024; kar-news</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
           <t>2026 report + older primary forms</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>2026 reported order; 2024 forms checked</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Government-subsidised seats including AIQ in checked undertaking; separate broad one-year Act form includes private/deemed/NRI/management categories.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="L5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Three years for the government-seat obligation. The March 2026 report describes credit for a completed one-year statutory service, leaving two additional years.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="N5" s="2" t="n">
         <v>5000000</v>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>Degree Rs50 lakh under the three-year undertaking; diploma Rs25 lakh separately. Current order and exact quota/cohort require confirmation.</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>Do not add one year plus three years automatically. The older broad one-year form exempts candidates who already completed qualifying MBBS compulsory rural service; confirm current Act, rules and exemptions.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="S5" s="2" t="inlineStr">
         <is>
           <t>Reported contract posting through counselling against vacancies, not a permanent-job guarantee. Current 2026 original order remains a gap.</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>kar-kea-forms2024; kar-news</t>
         </is>
@@ -972,56 +1798,79 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>1 year minimum</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Explicit AIQ: 2026 prospectus</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Government medical-college AIQ explicitly included in clause 11-1(b); continuous SR service for not less than one year. Conditional appointment/SS relief is separate.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>kerala-pg2026</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
           <t>2026 prospectus</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>General-merit/non-service government-medical-college PG entrants, including AIQ. Confirm private/self-financing seat applicability independently.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n">
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026 prospectus introduction and clause 11-1(b) expressly include AIQ candidates in government medical colleges. Self-financing colleges are covered only for admission procedures in the introduction.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>One continuous year immediately after completing the course, in the permitted government service roles.</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="N6" s="2" t="n">
         <v>5000000</v>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>Rs50 lakh bond; prospectus also calls for stipend/salary, government study expenditure and specified interest for failure of service. Rs50 lakh is not a verified all-inclusive cap.</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>Separate discontinuation bond and Rs50 lakh stray-vacancy damages provisions; do not treat these as the service obligation or automatically add all amounts.</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>In-service: ten years or up to superannuation, with separate salary-based damages. Annexures carry 2025–26 labels inside the 2026 PDF.</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>Relief for recognised SS degree; combined specialty/SS bonded service capped at two years under the clause. This relief explicitly excludes fellowship/observership. Certain regular public-service appointments have documentary release conditions.</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>In-service: ten years or up to superannuation, with separate salary-based damages. Annexures carry 2025–26 labels inside the 2026 PDF. Clause 11-1(c): relief for a regular Kerala/other-state/central/UT/qualifying PSU appointment if the appointing authority refuses joining-time extension; evidence and joining order within one month required. This is conditional relief, not an exemption at admission.</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>Clause 11-1(c): SS degree selection permits release to join; combined specialty/SS service capped at two years under those terms. This relief does not cover observership/fellowship. Do not assume a fellowship is an SS degree.</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
         <is>
           <t>Clause 11-1(k): absolution if government cannot offer qualifying work within one year after course completion. Obtain written discharge. Maternity clause describes a maximum 18-month stipendiary period including up to six months maternity leave; confirm the resulting completion date.</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="T6" s="2" t="inlineStr">
         <is>
           <t>kerala-pg2026</t>
         </is>
@@ -1045,56 +1894,79 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>1 year · older rule</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Goa Medical College 2020 PG amendment uploaded on MCC changes three years to one. Current continuation and original rule’s AIQ scope require the current college contract.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700479-BM</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
           <t>Older primary rule</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>2020 amendment; 2026 continuation unconfirmed</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Goa Medical College PG degree/diploma under the cited Goa University admission rules.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="L7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>2020 amendment changes PG government service from three years to one year.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="N7" s="2" t="n">
         <v>5000000</v>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>Rs50 lakh under the PG default/discontinuation clause. This is not the Rs1 crore neurosurgery superspecialty clause.</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>The same PG amendment describes Rs50 lakh for resignation/discontinuation as well; obtain the operative contract and triggers.</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>Historical institutional/state rule; not every institution in Goa.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>Government may permit higher-study deferment with Rs10 lakh degree / Rs7 lakh diploma bank guarantee, valid one year beyond studies; report back within a month.</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="S7" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="T7" s="2" t="inlineStr">
         <is>
           <t>mcc-700479-BM</t>
         </is>
@@ -1118,56 +1990,79 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Explicit AIQ: 2026 prospectus</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Government/municipal colleges; clause 20.4 expressly includes All India PG quota. Private unaided prohibition and AFMS obligations have separate scopes.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>maha-pg2026-brochure</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
           <t>2026 prospectus</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>NEET-PG 2026</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Government/municipal-corporation PG colleges; expressly both AIQ and state quota.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="L8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>One year social-responsibility service in a permitted employer category.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="N8" s="2" t="n">
         <v>5000000</v>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>Rs50 lakh for service default under clause 20.4.</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>Unaided private/minority seat resignation after the prescribed date: three years' fees. Government and special-institution exit terms need their applicable clause.</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>Clause 20.6 expressly says private unaided institutions shall not impose post-PG service bonds. Do not extend that exception to all deemed, central, trust or DNB institutions. In-service one-year medical-college service is additional to applicable DHS obligations.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="S8" s="2" t="inlineStr">
         <is>
           <t>Clause 20.5 lists permitted government/public employers within Maharashtra and Defence. Special institutions require their own contract.</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>maha-pg2026-brochure</t>
         </is>
@@ -1191,56 +2086,79 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>1 year · confirm cohort</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>GMC Bhopal MCC form: ordinary entrant one-year rural service. Form cites amendments through September 2025; confirm current college/year and private scope.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700296-BM</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
           <t>Primary form; cycle needs confirmation</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Form cites amendments through September 2025; year blank</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>GMC Bhopal MCC form: state/AIQ MD/MS; the form also explicitly describes execution for private-college entrants.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="L9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Ordinary non-in-service entrant: one year rural service.</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="N9" s="2" t="n">
         <v>1000000</v>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>Rs10 lakh ordinary-entrant rural-service default, as written in the checked form.</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>Government MD/MS seat-leaving form: Rs30 lakh after the prescribed cutoff; private-college form describes course/remaining-course tuition. Separate from Rs10 lakh service bond.</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="Q9" s="2" t="inlineStr">
         <is>
           <t>In-service: five years / Rs50 lakh. Exact 2026 private college/seat scope and amendments require confirmation; private does not automatically mean exempt.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="R9" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="S9" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="T9" s="2" t="inlineStr">
         <is>
           <t>mcc-700296-BM</t>
         </is>
@@ -1264,56 +2182,79 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>MAMC: 1 year; others vary</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Explicit AIQ: MAMC 2025–26 onwards</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>MAMC circular expressly includes AIQ and state quota. No uniform Delhi duration: UCMS, LHMC, VMMC, ABVIMS/RML need their own applicable policy.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>delhi-mamc-service-notice; du-pg2026; mcc-700122-BM</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
           <t>College-specific primary evidence</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>MAMC: 2025–26 onwards; DU exit form: 2026</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>MAMC MD/MS, both AIQ and state quota, under its 7 August 2025 circular. Other Delhi institutions require their own current policies.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="L10" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>MAMC: minimum one year in GNCT Delhi health facilities immediately after course completion.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="N10" s="2" t="n">
         <v>2000000</v>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>MAMC PG service bond Rs20 lakh. Annexure has both 12% interest wording and a stated total-obligation cap; confirm the current PG-specific form rather than assuming an all-inclusive payable amount.</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>DU MD/MS: separate Rs10 lakh surety for specified surrender, course-leaving or cancellation triggers. VMMC/GGSIPU undated form: separate Rs3 lakh exit surety; confirm year. These are not annual fees.</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="Q10" s="2" t="inlineStr">
         <is>
           <t>Delhi is not uniformly free of bonds. DU affiliation does not remove a college service circular. Do not export MAMC rules to AIIMS, central MoHFW colleges, UCMS, LHMC, VMMC or RML without their own authority/cohort evidence.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t>No blanket SS/fellowship waiver established. MAMC also names SS students; verify deferment and any cumulative obligation for an MD/MS entrant.</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="S10" s="2" t="inlineStr">
         <is>
           <t>MAMC notice states the minimum service and admission-year scope. Current written posting/pay/release conditions remain essential.</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="T10" s="2" t="inlineStr">
         <is>
           <t>delhi-mamc-service-notice; du-pg2026; du-surety2026; mcc-700122-BM</t>
         </is>
@@ -1337,54 +2278,79 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026 rule; terms incomplete</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+          <t>2 years · confirm cohort</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>SCB government-college bond supplied on MCC specifies two years; AIQ not separately named and year blank. January 2026 placement guidance corroborates two years for a graduating cohort.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700336-BM; odisha-postpg-guidelines2026; odisha-pg2026-guidelines</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>2026 guideline + undated college form</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>2026–27</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>DMET guideline J(5) requires a service bond except for candidates opting for private medical colleges.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Service-bond submission confirmed; ordinary entrant's full duration not established from the checked operative terms.</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Numeric post-PG default formula not established; do not substitute the Rs10 lakh exit penalty.</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Two years in the checked SCB government-college service bond. Placement guidance counts the two-year posting as SR; relevant peripheral rotation is included within it.</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>SCB Annexure A: twice the stipend/salary received for three years of study. Variable formula, not a fixed Rs10 lakh service bond; Rs10 lakh is the separate course-exit principal.</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>J(3): Rs10 lakh plus stipend/salary refund; fees not refunded, under the specified exit conditions.</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Private-college exception to J(5) is explicit. In-service M(4) two-year wording must not be used as proof of an ordinary entrant's duration. Central AIIMS and DNB require their own rules.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>Not established from the checked material; obtain the current college/order clause.</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>Not established from the checked material; obtain the current college/order clause.</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>odisha-pg2026-guidelines</t>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>2026 guideline J(5) excepts private medical colleges from that service-bond submission. Pre/para-clinical placement in medical colleges is not a service exemption. AIIMS/INI and private/DNB contracts need their own applicable rules; do not assign the government MD/MS rule by geography alone.</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>SCB form: recognised higher study temporarily suspends the bond, which resumes after completion. Its definition excludes outside-state residency/fellowship.</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>Join within 30 days of receipt of appointment in the SCB form. Qualifying government work inside Odisha counts. No verified automatic no-posting release deadline.</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>odisha-pg2026-guidelines; mcc-700336-BM; odisha-postpg-guidelines2026</t>
         </is>
       </c>
     </row>
@@ -1406,52 +2372,69 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>Campus / route unresolved</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Current AIQ terms unresolved</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Separate a genuine state-government MD/MS AIQ seat from deemed paid seats and DNB. JIPMER MD/MS is an INI-CET route outside this MCC AIQ table. No current universal zero-year finding.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
           <t>Unresolved</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Current MD/MS terms not established</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>State-government, private/deemed and central JIPMER are separate admission/employment systems.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>No current state/campus-specific post-MD/MS service rule verified in this research.</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="Q12" s="2" t="inlineStr">
         <is>
           <t>No verified rule is not a finding of no bond. JIPMER uses its own INI-CET prospectus/contract; do not assume the UT government rule governs it.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="R12" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="S12" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1471,56 +2454,79 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>3 years · older rule</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>RIMS Ranchi MCC-uploaded 2018 resolution. Confirm current RIMS/other state-college AIQ contract; this is not a rule for central AIIMS Deoghar.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700418-BM</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
           <t>Older primary rule</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>2018 resolution cited; 2026 continuation unconfirmed</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>RIMS Ranchi PG bond form; verify latest institution/state conditions.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="L13" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Three years government service in the checked RIMS form.</t>
         </is>
       </c>
-      <c r="I13" s="2" t="n">
+      <c r="N13" s="2" t="n">
         <v>3000000</v>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>Rs30 lakh plus stipend and other payments during the course under the checked service-default resolution.</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="P13" s="2" t="inlineStr">
         <is>
           <t>Non-joining/discontinuation clauses also contain Rs30 lakh liability; get separate exact trigger and repayment wording.</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="Q13" s="2" t="inlineStr">
         <is>
           <t>Do not assign this RIMS/state rule to AIIMS Deoghar or every private/DNB institution.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="R13" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="S13" s="2" t="inlineStr">
         <is>
           <t>Form says bond ceases if state appointment is not made within six months after passing. Confirm the current rule and written discharge.</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="T13" s="2" t="inlineStr">
         <is>
           <t>mcc-700418-BM</t>
         </is>
@@ -1544,54 +2550,79 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>2 years · confirm cohort</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Dr SN Jodhpur non-service form explicitly names AIQ. The page with five years is in-service. Values differ by branch; other campus/current relief orders require checking.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700308-BM; mcc-sms-bond</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
           <t>Primary form; cycle needs confirmation</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>SMS pack / specialty-value order: 2025–26</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>SMS Jaipur pack labels MD/MS service bond for AIQ and state-quota PG students. Values differ by specialty.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Duration not established from the specialty-value order; obtain current service undertaking.</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Dr SN Jodhpur undertaking expressly covers AIQ and state non-service MD/MS entrants in government, government-society and RUHS colleges; confirm each campus/current cohort.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Two years for AIQ/state non-service entrants, explicit in Dr SN Jodhpur service undertaking p.2. Five years on p.3 belongs to the separate in-service form.</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>2025 table: Radiodiagnosis/Dermatology/Medicine/OBG Rs1.5 crore; Ophthalmology/Paediatrics/General Surgery (and listed others) Rs1 crore; ENT/Radiation Oncology/Pathology/Nuclear Medicine/Palliative Medicine (and others) Rs50 lakh; Biochemistry/Pharmacology (and others) Rs25 lakh.</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="P14" s="2" t="inlineStr">
         <is>
           <t>Separate course-exit surety Rs10 lakh. A Rs1.5 lakh bank guarantee / Rs8.5 lakh surety split appears in the pack; it is not the branch-specific service bond.</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="Q14" s="2" t="inlineStr">
         <is>
           <t>The displayed service amounts are from a 2025 order, not a verified unchanged 2026 schedule. Do not use one statewide Rs25 lakh default for all branches.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="R14" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="S14" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>mcc-sms-bond</t>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>mcc-sms-bond; mcc-700308-BM</t>
         </is>
       </c>
     </row>
@@ -1613,56 +2644,79 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>2 years · older rule</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>State government/autonomous colleges under the KGMU form citing the 2018 order. Central BHU/AMU, AIIMS and private/DNB are separate; geography does not transfer this bond.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700366-BM</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
           <t>Older primary rule</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>2018 order cited; 2026 continuation unconfirmed</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>KGMU form names state government/autonomous MD/MS institutions under the cited UP order.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="L15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Two years government service under the checked form.</t>
         </is>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="N15" s="2" t="n">
         <v>4000000</v>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="O15" s="2" t="inlineStr">
         <is>
           <t>MD/MS Rs40 lakh; diploma Rs20 lakh separately.</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="P15" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="Q15" s="2" t="inlineStr">
         <is>
           <t>Do not apply a state KGMU form automatically to central BHU, AIIMS or private/DNB institutions.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="R15" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="S15" s="2" t="inlineStr">
         <is>
           <t>Historical order clause 2(6): release if not posted within three months of successful completion; it also describes deferment when selected for a higher course. Obtain current written rules before relying on either.</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
+      <c r="T15" s="2" t="inlineStr">
         <is>
           <t>mcc-700366-BM</t>
         </is>
@@ -1686,54 +2740,77 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>2 years · scheme dependent</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Conditional subsidised-fee scheme</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Older undertaking expressly includes Central quota but links service to opting for subsidised tuition. Mixed Doon/Haldwani documents do not establish a universal current two-year obligation or exemption for full-fee seats.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700386-BM</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
           <t>Conflicting older forms</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Mixed 2021–22 / 2017-linked schemes; 2026 unresolved</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Mixed MCC attachment contains a Doon 2021–22 form and a separate optional subsidised-fee scheme; it is not one clean current Haldwani policy.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="L16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Both older schemes describe two years in government facilities in hilly areas, conditional on the applicable scheme.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" s="2" t="inlineStr">
         <is>
           <t>Conflicting formulas: Doon 2021–22 Rs2.5 crore; subsidised-fee scheme full-course fees less fees paid plus compound interest. No single verified 2026 principal assigned.</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="P16" s="2" t="inlineStr">
         <is>
           <t>Discontinuation also has scheme-specific liability; obtain the actual current selected-fee-route contract.</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="Q16" s="2" t="inlineStr">
         <is>
           <t>Check whether service bond is linked to an optional subsidised tuition route and whether an earlier MBBS bond adds obligations. Do not use a historical amount as a current universal rule.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="R16" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="S16" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="T16" s="2" t="inlineStr">
         <is>
           <t>mcc-700386-BM</t>
         </is>
@@ -1757,56 +2834,81 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>3 years · confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Three years corroborated by 2026 open/non-service bulletin and Burdwan MCC bond. Confirm college AIQ cohort; open means non-in-service, not only UR reservation.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>wb-pg2026-bulletin; mcc-700388-BM</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
           <t>2026 rule; terms incomplete</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Open/non-in-service category under WBMCC clause 12, subject to government order and institution applicability.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="L17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>PG degree: three years; PG diploma: two years is a separate qualification.</t>
         </is>
       </c>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>Penalty as fixed by government; numeric service-default amount not established from this bulletin.</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>Burdwan MCC form: Rs10 lakh per defaulting year; three wholly unserved years imply Rs30 lakh principal under that form. Current college formula/cohort must be confirmed; not a universal all-inclusive demand.</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>PG degree discontinuation Rs5 lakh; diploma Rs2 lakh. Bulletin says no DNB discontinuation bond at present; that does not establish no DNB post-course service bond.</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="Q17" s="2" t="inlineStr">
         <is>
           <t>In-service TR rules are separate. Open category is not synonymous with unreserved caste category. Confirm private/deemed/AIQ and institution-specific scope before applying.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="R17" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="S17" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>wb-pg2026-bulletin</t>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>wb-pg2026-bulletin; mcc-700388-BM</t>
         </is>
       </c>
     </row>
@@ -1828,54 +2930,77 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>2 years · 2025 form</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Pt JNM Raipur form expressly includes AIQ/state, cites November 2025 gazette and fills admission year 2025. Confirm current form; do not apply to AIIMS Raipur.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>mcc-raipur-bond</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
           <t>Primary form; cycle needs confirmation</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>November 2025 gazette / 2025 joining form</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Pt JNM Raipur form describes state/AIQ and general/reserved entrants to government MD/MS.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="L18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Two years of state government service in the checked form.</t>
         </is>
       </c>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="n"/>
+      <c r="O18" s="2" t="inlineStr">
         <is>
           <t>Principal penalty field is blank in the upload; stipend recovery is stated. Amount must be obtained from the applicable notification/category, not guessed.</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="P18" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="Q18" s="2" t="inlineStr">
         <is>
           <t>Current admission year/category terms need confirmation; no automatic application to central AIIMS Raipur or private/DNB institutions.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="R18" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="S18" s="2" t="inlineStr">
         <is>
           <t>Form clause 9 says bond automatically ceases if appointment order not issued within twelve months after the university completion information is received. Verify the precise current trigger and obtain discharge.</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="T18" s="2" t="inlineStr">
         <is>
           <t>mcc-raipur-bond</t>
         </is>
@@ -1899,74 +3024,97 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
+          <t>3 years · 2025 prospectus</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>College / older rule: confirm AIQ cohort</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>State-government PG bonds in 2025 prospectus. Specified already-government-employed AIQ entrants have a 2019 exception; ordinary AIQ admission alone is not that exception.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>bihar-pg2025</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
           <t>2025 prospectus</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>2025 with incorporated 2017/2019 resolutions</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>State-government medical-college PG entrants covered by Annexure 4 resolutions.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="L19" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Three years under the state government after PG completion.</t>
         </is>
       </c>
-      <c r="I19" s="2" t="n">
+      <c r="N19" s="2" t="n">
         <v>2500000</v>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>Rs25 lakh plus salary received in the service period under the checked resolution; not a verified all-inclusive cap.</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="P19" s="2" t="inlineStr">
         <is>
           <t>Rs15 lakh plus stipend for leaving the PG course under the checked resolution.</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="Q19" s="2" t="inlineStr">
         <is>
           <t>2019 relief is for specified AIQ entrants already employed by central/other-state government or an instrumentality. It is not a general AIQ exemption. 2026 continuation must be checked.</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="R19" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="S19" s="2" t="inlineStr">
         <is>
           <t>Not established from the checked material; obtain the current college/order clause.</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="T19" s="2" t="inlineStr">
         <is>
           <t>bihar-pg2025</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O19"/>
+  <autoFilter ref="A1:T19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2089,13 +3237,183 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh government colleges: State/CQ versus AIQ</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>The current NTRUHS Annexure A is explicitly State/CQ, one year / Rs40 lakh. It does not establish that obligation for an AIQ entrant. Ask the chosen college for its AIQ service order; no positive AIQ exemption is claimed either.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ap-cq2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>SVIMS Tirupati</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>The AP prospectus expressly assigns SVIMS its own tuition, training, stipend, bonds and service norms. Do not substitute the general AP State/CQ rule or label it bond-free without the SVIMS current admission contract.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ap-cq2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Gandhi Secunderabad / Osmania Hyderabad</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>MCC college bonds support one-year service if required. Gandhi form is 2025–26; Osmania service form is 2023–24. Confirm 2026–27 execution. A Rs50 lakh course-exit bond is distinct from Rs20 lakh MD/MS service liability.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700481-BM; mcc-700483-BM; ts-cq2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Kerala government colleges: conditional relief</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>AIQ is expressly included in the one-year requirement. Qualifying regular government/PSU appointment can permit release if joining-time extension is refused, with documentary conditions. SS degree relief exists; fellowship/observership is excluded from that relief.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>kerala-pg2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Odisha private colleges / government pre- and para-clinical departments</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026 admission guideline J(5) excepts private colleges from that bond-submission clause. In government colleges, pre/para-clinical doctors are assigned to medical colleges rather than the peripheral rotation; this is a placement distinction, not abolition of the two-year bond.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>odisha-pg2026-guidelines; mcc-700336-BM; odisha-postpg-guidelines2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Dr SN Jodhpur / Rajasthan state and society colleges</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>AIQ non-service undertaking specifies two years. Its separate 2026–27 five-year / Rs80 lakh form is for in-service candidates. SMS 2025 branch values range Rs25 lakh to Rs1.5 crore. Do not transfer an outdated flat Rs25 lakh to every branch or assume an unverified government-job waiver.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700308-BM; mcc-sms-bond</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>BHU / AMU and other central institutions in Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>The UP state-college two-year bond is not evidence for a central university. BHU’s checked 2025 junior-resident agreement concerns the three-year training and course-exit damages; it is not an affirmative current no-service certificate. Obtain the central institution’s own contract.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700366-BM; mcc-bhu-bond</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Uttarakhand government colleges: subsidised tuition option</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Older Central/state-quota undertaking links two years of hill service to a subsidised-fee option. Its separate Doon form has different financial terms. Obtain the chosen campus’s current full-fee and subsidised-fee terms; do not assign historical fees, penalties or a zero-year option to every campus.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700386-BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Bihar: already-government-employed AIQ entrants</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2019 resolution describes a limited exception for AIQ entrants already employed by central/other-state government or an instrumentality. It is not an exemption for an ordinary applicant simply joining via AIQ.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>bihar-pg2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>AFMS institutions / AFMC Pune: Priority-V civilian PG entrants</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Separate AFMS route in MCC bulletin: five years of Armed Forces service on Short Service Commission, subject to commissioning/medical and age conditions. The checked bond specifies Rs60.5 lakh plus applicable interest under its default triggers. Do not replace this with Maharashtra’s ordinary one-year bond.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>mcc-bulletin2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C7"/>
+  <autoFilter ref="A1:C17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2226,13 +3544,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2585,7 +3903,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>PDF p.12 section 5; in-service pp.10–11; SVIMS p.18; exit p.19</t>
+          <t>PDF p.29 Annexure A State/CQ-specific bond; p.12 section 5; in-service pp.10–11; SVIMS p.18; exit p.19</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -2595,13 +3913,13 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>maximum period of 18 months; penalty of Rs.40,00,000</t>
+          <t>maximum period of 18 months; penalty of Rs.40,00,000; State Quota/Competent Authority Quota seats</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Section 13.2 has a PG Dental wording carryover in this medical prospectus. Exit amount is therefore not treated as an unqualified MD/MS confirmation; SVIMS has separate appended terms.</t>
+          <t>Annexure A explicitly limits the one-year bond to State/CQ seats: not verified AIQ scope or a positive AIQ exemption. Section 13.2 has a PG Dental wording carryover; SVIMS has separate terms.</t>
         </is>
       </c>
     </row>
@@ -2755,7 +4073,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>PDF pp.35–38 clauses 11–12; Annexure XV pp.74–76 and XVI pp.77–79</t>
+          <t>Introduction; PDF pp.35–38 clauses 11–12, including explicit AIQ clause 11-1(b) and relief 11-1(c); Annexure XV pp.74–76 and XVI pp.77–79</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -2813,7 +4131,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>PDF p.47 clauses 20.3–20.7; private unaided circular Annexure X</t>
+          <t>PDF p.47 clause 20.4 expressly covers AIQ/state, 20.5 permitted service, 20.6 private unaided exception; Annexure X</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -3587,13 +4905,481 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>mcc-bulletin2026</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>MCC NEET-PG counselling information bulletin 2026</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Medical Counselling Committee / DGHS</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://cdnbbsr.s3waas.gov.in/s3e0f7a4d0ef9b84b83b693bbf3feb8e6e/uploads/2026/10/202610082121348550.pdf</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>c3fd152169d36fc74c6ac17ab40f66836e2eb5e877bf7b56b527529f25048564</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>PDF p.7 clause 2.14; p.41 DNB; p.57 FAQ 23; pp.119–122 AFMS bond</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Official publication</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>may vary from State to State and Institute to Institute; to serve for 05 years</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>MCC counselling includes AIQ, central, deemed and DNB routes. AFMS Priority-V civilian service is a distinct route, not the ordinary state AIQ bond. PDF carries a draft-version label on its cover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700481-BM</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Gandhi Medical College Secunderabad PG bond forms on MCC</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Gandhi Medical College / Telangana DME</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>2025–26 college form on 2026 MCC portal</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700481&amp;Type=BM</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>39c98e501441548ce34f8ee3efc20e6878d28343f398f8effbf48fad7bf5c6b9</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>PDF p.3 Annexure II, for all candidates; p.4 service sureties; pp.1–2 exit bond</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Official publication</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>year202 5-26; maximum period of18 month; 20,00,000</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Page 3 visually checked: all candidates, one year as SR if required, within 18 months, Rs20 lakh MD/MS.</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>College upload supports a one-year planning assumption for this AIQ college; the form is dated 2025–26. Obtain its 2026–27 replacement; it does not independently establish every Telangana campus contract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700483-BM</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Osmania Medical College PG bond forms on MCC</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Osmania Medical College / Telangana DME</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2023–24 form on 2026 MCC portal</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700483&amp;Type=BM</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>c7b90e8cb66d9c2de260a556c77c8cc43a4edf08092d0e947b46f635c52eb7db</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>PDF pp.3–4 service agreement; p.1 separate Rs50 lakh exit undertaking</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Official publication</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Pages 3–4 visually reviewed: 2023–24, one year for non-service candidates, Rs20 lakh PG degree / Rs10 lakh diploma; GO155 dated 18 November 2021.</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Historical college form; do not call its portal retrieval date the admission year. Supports the service obligation, not a verified 2026 signed contract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700336-BM</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>SCB Medical College Cuttack government service bond on MCC</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>SCB Medical College / Government of Odisha</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Undated form on 2026 MCC portal</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700336&amp;Type=BM</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>e0eab29378165f9ee1abe494bfb91320244be72a3f9143c88246ad9318eae858</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>PDF pp.1–3 Annexure A: two-year service, double-stipend default, higher study and qualifying work</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Official publication</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>All three pages visually reviewed: two years after completion; default twice three years of stipend/salary; join within 30 days of appointment. Higher study temporarily suspends the bond; outside-state residency/fellowship excluded from that definition. Qualifying state-government work inside Odisha counts.</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Admission-year field is blank and AIQ is not named separately; this is a government-college form published for MCC candidates. Confirm current college execution. Not an Odisha private/deemed/central blanket rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>odisha-postpg-guidelines2026</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Odisha post-PG bonded doctor placement notification</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Odisha Health &amp; Family Welfare Department / DMET</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Posted in January 2026 for the 2022 admission batch</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://dmetodisha.in/POST_PG_Static/DOWNLOADSPGM_22/GUIDELINES FOR POST PG BOND SR DOCTORS_02_01_2026.pdf</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>4879a5364cf3bf450f724c9ff932c7fe5c728674375d7c556d3b39ed7b218936</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>PDF p.1 clauses 1–5; two-year SR placement and one-year peripheral rotation</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Official publication</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>duration of 2 years Post PG posting; excluding the Superspecialist and pre and para clinical doctors</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Placement guidance for a graduating cohort, not a standalone 2026 entrant contract. One-year peripheral deployment is within the two-year obligation; do not add it as a third year. Pre/para-clinical doctors are posted in medical colleges, not exempted from all service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700308-BM</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Dr SN Medical College Jodhpur AIQ/state PG service undertaking</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Dr SN Medical College / Government of Rajasthan</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Mixed forms on 2026 MCC portal; non-service year blank</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700308&amp;Type=BM</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>32c800e03f4f29110318d3578150cc107e636fc86309504a28060ad7c4e77e79</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>PDF p.2 AIQ/state non-service undertaking clause 1; p.3 separate 2026–27 in-service form</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Official publication</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>FOR ALL INDIA QUOTA &amp; STATE QUOTA (NON SERVICE); period of two year; 2026-2027</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Two years is explicit for non-service entrants. The five-year clause on p.3 is for in-service entrants. Four specialty-dependent default amounts are listed; obtain current branch allocation and any subsequent relief order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>mcc-700388-BM</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Burdwan Medical College PG exit and service bond on MCC</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Burdwan Medical College / Government of West Bengal</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Undated form citing 2013/2014 notifications</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700388&amp;Type=BM</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>1d49448163592ff63a80cbf1ac3821158ed1eeca62ac95dbc4ca24a10b1333fd</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>PDF p.2 indemnity for non-sponsored trainees; p.1 separate exit undertaking</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Official publication</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 visually reviewed: three continuous years; Rs10 lakh for each defaulting year; names state medical teaching institutions and SR designation. Page 1 exit: Rs5 lakh degree / Rs2 lakh diploma.</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>MCC college-upload evidence for AIQ planning; year blank and older orders cited. Current WBMCC bulletin corroborates three years but a current college AIQ contract still needs checking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>mcc-bhu-bond</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>BHU agreement for MD/MS/MDS junior residents on MCC</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Institute of Medical Sciences, Banaras Hindu University</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>2025 agreement</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://mcc.admissions.nic.in/Applicant/Handler/ViewInstituteProfileDynamic.ashx?boardId=140012621&amp;InstituteId=700323&amp;Type=BM</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>61c738aaebca9a3f5a64ac20a17f9d59dc833cc5de7ca994d3e816d90c48b08f</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>PDF pp.1–7, especially p.5 clause 12 course exit; full agreement checked</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Official publication</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>liquidated damages; 2025</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Three-year training appointment and Rs5 lakh course-exit damages. Silence on a separate post-PG service policy is not affirmative proof of exemption or zero years.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L23"/>
+  <autoFilter ref="A1:L31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>